<commit_message>
task 06 & 07
</commit_message>
<xml_diff>
--- a/Excel/PracticeExcel/02Functions_Formulas/sample-data-fx.blank.xlsx
+++ b/Excel/PracticeExcel/02Functions_Formulas/sample-data-fx.blank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 7490\Documents\PythonClassSF\DataAnalytics01\Excel\02Functions_Formulas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF60EF9A-8E98-425F-BFB5-280FCDC9DB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F724FB2C-EACB-470B-9067-2343E8D16EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="6" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{26D4546B-D2A1-4444-8EAF-A6228F96F0C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,8 @@
     <sheet name="Task 03" sheetId="5" r:id="rId5"/>
     <sheet name="Task 04" sheetId="6" r:id="rId6"/>
     <sheet name="Task 05" sheetId="7" r:id="rId7"/>
+    <sheet name="Task 06" sheetId="8" r:id="rId8"/>
+    <sheet name="Task 07" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -64,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2437" uniqueCount="787">
   <si>
     <t>Essential Excel Functions &amp; Formulas</t>
   </si>
@@ -2404,6 +2406,27 @@
   </si>
   <si>
     <t>Count:</t>
+  </si>
+  <si>
+    <t>Employee Id</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>First name</t>
+  </si>
+  <si>
+    <t>Last name</t>
+  </si>
+  <si>
+    <t>Entire Data horizantally</t>
+  </si>
+  <si>
+    <t>Entire Data Vertically</t>
+  </si>
+  <si>
+    <t>Entire All Data Get by last name using Filter</t>
   </si>
 </sst>
 </file>
@@ -2466,7 +2489,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2500,6 +2523,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2554,7 +2583,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2633,6 +2662,11 @@
     </xf>
     <xf numFmtId="165" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2676,8 +2710,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="5" name="">
@@ -2696,7 +2730,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="5" name="">
@@ -2751,6 +2785,7 @@
           <inkml:channelProperty channel="OE" name="resolution" value="1000" units="1/deg"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-05-22T01:50:00.741"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.1" units="cm"/>
@@ -2763,7 +2798,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71B18D4F-F180-46A4-9272-AD02F8205A18}" name="staff" displayName="staff" ref="C7:O267" totalsRowShown="0">
-  <autoFilter ref="C7:O267" xr:uid="{71B18D4F-F180-46A4-9272-AD02F8205A18}"/>
+  <autoFilter ref="C7:O267" xr:uid="{71B18D4F-F180-46A4-9272-AD02F8205A18}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Tuxwell"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C8:O267">
     <sortCondition ref="C7:C267"/>
   </sortState>
@@ -4616,7 +4657,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" hidden="1">
       <c r="C8" t="s">
         <v>42</v>
       </c>
@@ -4657,7 +4698,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" hidden="1">
       <c r="C9" t="s">
         <v>51</v>
       </c>
@@ -4780,7 +4821,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" hidden="1">
       <c r="C12" t="s">
         <v>61</v>
       </c>
@@ -4821,7 +4862,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" hidden="1">
       <c r="C13" t="s">
         <v>68</v>
       </c>
@@ -4862,7 +4903,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" hidden="1">
       <c r="C14" t="s">
         <v>72</v>
       </c>
@@ -4903,7 +4944,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" hidden="1">
       <c r="C15" t="s">
         <v>75</v>
       </c>
@@ -4944,7 +4985,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" hidden="1">
       <c r="C16" t="s">
         <v>79</v>
       </c>
@@ -4985,7 +5026,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="3:15">
+    <row r="17" spans="3:15" hidden="1">
       <c r="C17" t="s">
         <v>83</v>
       </c>
@@ -5026,7 +5067,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="3:15">
+    <row r="18" spans="3:15" hidden="1">
       <c r="C18" t="s">
         <v>87</v>
       </c>
@@ -5067,7 +5108,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="3:15">
+    <row r="19" spans="3:15" hidden="1">
       <c r="C19" t="s">
         <v>90</v>
       </c>
@@ -5108,7 +5149,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="3:15">
+    <row r="20" spans="3:15" hidden="1">
       <c r="C20" t="s">
         <v>94</v>
       </c>
@@ -5149,7 +5190,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="3:15">
+    <row r="21" spans="3:15" hidden="1">
       <c r="C21" t="s">
         <v>98</v>
       </c>
@@ -5190,7 +5231,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="3:15">
+    <row r="22" spans="3:15" hidden="1">
       <c r="C22" t="s">
         <v>102</v>
       </c>
@@ -5231,7 +5272,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="3:15">
+    <row r="23" spans="3:15" hidden="1">
       <c r="C23" t="s">
         <v>106</v>
       </c>
@@ -5272,7 +5313,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="3:15">
+    <row r="24" spans="3:15" hidden="1">
       <c r="C24" t="s">
         <v>110</v>
       </c>
@@ -5313,7 +5354,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="3:15">
+    <row r="25" spans="3:15" hidden="1">
       <c r="C25" t="s">
         <v>113</v>
       </c>
@@ -5354,7 +5395,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="3:15">
+    <row r="26" spans="3:15" hidden="1">
       <c r="C26" t="s">
         <v>117</v>
       </c>
@@ -5395,7 +5436,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="3:15">
+    <row r="27" spans="3:15" hidden="1">
       <c r="C27" t="s">
         <v>120</v>
       </c>
@@ -5436,7 +5477,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="3:15">
+    <row r="28" spans="3:15" hidden="1">
       <c r="C28" t="s">
         <v>124</v>
       </c>
@@ -5477,7 +5518,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="3:15">
+    <row r="29" spans="3:15" hidden="1">
       <c r="C29" t="s">
         <v>127</v>
       </c>
@@ -5518,7 +5559,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="3:15">
+    <row r="30" spans="3:15" hidden="1">
       <c r="C30" t="s">
         <v>130</v>
       </c>
@@ -5559,7 +5600,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="3:15">
+    <row r="31" spans="3:15" hidden="1">
       <c r="C31" t="s">
         <v>133</v>
       </c>
@@ -5600,7 +5641,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="3:15">
+    <row r="32" spans="3:15" hidden="1">
       <c r="C32" t="s">
         <v>133</v>
       </c>
@@ -5641,7 +5682,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="3:15">
+    <row r="33" spans="3:15" hidden="1">
       <c r="C33" t="s">
         <v>136</v>
       </c>
@@ -5682,7 +5723,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="3:15">
+    <row r="34" spans="3:15" hidden="1">
       <c r="C34" t="s">
         <v>139</v>
       </c>
@@ -5723,7 +5764,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="3:15">
+    <row r="35" spans="3:15" hidden="1">
       <c r="C35" t="s">
         <v>142</v>
       </c>
@@ -5764,7 +5805,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="36" spans="3:15">
+    <row r="36" spans="3:15" hidden="1">
       <c r="C36" t="s">
         <v>146</v>
       </c>
@@ -5805,7 +5846,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="3:15">
+    <row r="37" spans="3:15" hidden="1">
       <c r="C37" t="s">
         <v>149</v>
       </c>
@@ -5846,7 +5887,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="3:15">
+    <row r="38" spans="3:15" hidden="1">
       <c r="C38" t="s">
         <v>152</v>
       </c>
@@ -5887,7 +5928,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="3:15">
+    <row r="39" spans="3:15" hidden="1">
       <c r="C39" t="s">
         <v>156</v>
       </c>
@@ -5928,7 +5969,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="3:15">
+    <row r="40" spans="3:15" hidden="1">
       <c r="C40" t="s">
         <v>159</v>
       </c>
@@ -5969,7 +6010,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="41" spans="3:15">
+    <row r="41" spans="3:15" hidden="1">
       <c r="C41" t="s">
         <v>162</v>
       </c>
@@ -6010,7 +6051,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="3:15">
+    <row r="42" spans="3:15" hidden="1">
       <c r="C42" t="s">
         <v>165</v>
       </c>
@@ -6051,7 +6092,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="3:15">
+    <row r="43" spans="3:15" hidden="1">
       <c r="C43" t="s">
         <v>168</v>
       </c>
@@ -6092,7 +6133,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="44" spans="3:15">
+    <row r="44" spans="3:15" hidden="1">
       <c r="C44" t="s">
         <v>171</v>
       </c>
@@ -6133,7 +6174,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="45" spans="3:15">
+    <row r="45" spans="3:15" hidden="1">
       <c r="C45" t="s">
         <v>174</v>
       </c>
@@ -6174,7 +6215,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="46" spans="3:15">
+    <row r="46" spans="3:15" hidden="1">
       <c r="C46" t="s">
         <v>177</v>
       </c>
@@ -6215,7 +6256,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="47" spans="3:15">
+    <row r="47" spans="3:15" hidden="1">
       <c r="C47" t="s">
         <v>180</v>
       </c>
@@ -6256,7 +6297,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="48" spans="3:15">
+    <row r="48" spans="3:15" hidden="1">
       <c r="C48" t="s">
         <v>183</v>
       </c>
@@ -6297,7 +6338,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="3:15">
+    <row r="49" spans="3:15" hidden="1">
       <c r="C49" t="s">
         <v>186</v>
       </c>
@@ -6338,7 +6379,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="3:15">
+    <row r="50" spans="3:15" hidden="1">
       <c r="C50" t="s">
         <v>189</v>
       </c>
@@ -6379,7 +6420,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="3:15">
+    <row r="51" spans="3:15" hidden="1">
       <c r="C51" t="s">
         <v>192</v>
       </c>
@@ -6420,7 +6461,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="3:15">
+    <row r="52" spans="3:15" hidden="1">
       <c r="C52" t="s">
         <v>192</v>
       </c>
@@ -6461,7 +6502,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="3:15">
+    <row r="53" spans="3:15" hidden="1">
       <c r="C53" t="s">
         <v>197</v>
       </c>
@@ -6502,7 +6543,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="3:15">
+    <row r="54" spans="3:15" hidden="1">
       <c r="C54" t="s">
         <v>200</v>
       </c>
@@ -6543,7 +6584,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="3:15">
+    <row r="55" spans="3:15" hidden="1">
       <c r="C55" t="s">
         <v>203</v>
       </c>
@@ -6584,7 +6625,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="56" spans="3:15">
+    <row r="56" spans="3:15" hidden="1">
       <c r="C56" t="s">
         <v>206</v>
       </c>
@@ -6666,7 +6707,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="3:15">
+    <row r="58" spans="3:15" hidden="1">
       <c r="C58" t="s">
         <v>210</v>
       </c>
@@ -6707,7 +6748,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="3:15">
+    <row r="59" spans="3:15" hidden="1">
       <c r="C59" t="s">
         <v>213</v>
       </c>
@@ -6748,7 +6789,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="60" spans="3:15">
+    <row r="60" spans="3:15" hidden="1">
       <c r="C60" t="s">
         <v>216</v>
       </c>
@@ -6789,7 +6830,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="61" spans="3:15">
+    <row r="61" spans="3:15" hidden="1">
       <c r="C61" t="s">
         <v>220</v>
       </c>
@@ -6830,7 +6871,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="62" spans="3:15">
+    <row r="62" spans="3:15" hidden="1">
       <c r="C62" t="s">
         <v>223</v>
       </c>
@@ -6871,7 +6912,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="63" spans="3:15">
+    <row r="63" spans="3:15" hidden="1">
       <c r="C63" t="s">
         <v>226</v>
       </c>
@@ -6912,7 +6953,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="64" spans="3:15">
+    <row r="64" spans="3:15" hidden="1">
       <c r="C64" t="s">
         <v>229</v>
       </c>
@@ -6953,7 +6994,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="65" spans="3:15">
+    <row r="65" spans="3:15" hidden="1">
       <c r="C65" t="s">
         <v>232</v>
       </c>
@@ -6994,7 +7035,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="3:15">
+    <row r="66" spans="3:15" hidden="1">
       <c r="C66" t="s">
         <v>235</v>
       </c>
@@ -7035,7 +7076,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="67" spans="3:15">
+    <row r="67" spans="3:15" hidden="1">
       <c r="C67" t="s">
         <v>238</v>
       </c>
@@ -7076,7 +7117,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="68" spans="3:15">
+    <row r="68" spans="3:15" hidden="1">
       <c r="C68" t="s">
         <v>241</v>
       </c>
@@ -7117,7 +7158,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="69" spans="3:15">
+    <row r="69" spans="3:15" hidden="1">
       <c r="C69" t="s">
         <v>244</v>
       </c>
@@ -7158,7 +7199,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="3:15">
+    <row r="70" spans="3:15" hidden="1">
       <c r="C70" t="s">
         <v>247</v>
       </c>
@@ -7199,7 +7240,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="71" spans="3:15">
+    <row r="71" spans="3:15" hidden="1">
       <c r="C71" t="s">
         <v>248</v>
       </c>
@@ -7240,7 +7281,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="72" spans="3:15">
+    <row r="72" spans="3:15" hidden="1">
       <c r="C72" t="s">
         <v>251</v>
       </c>
@@ -7281,7 +7322,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="3:15">
+    <row r="73" spans="3:15" hidden="1">
       <c r="C73" t="s">
         <v>254</v>
       </c>
@@ -7322,7 +7363,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="74" spans="3:15">
+    <row r="74" spans="3:15" hidden="1">
       <c r="C74" t="s">
         <v>257</v>
       </c>
@@ -7363,7 +7404,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="75" spans="3:15">
+    <row r="75" spans="3:15" hidden="1">
       <c r="C75" t="s">
         <v>260</v>
       </c>
@@ -7404,7 +7445,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="76" spans="3:15">
+    <row r="76" spans="3:15" hidden="1">
       <c r="C76" t="s">
         <v>260</v>
       </c>
@@ -7445,7 +7486,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="77" spans="3:15">
+    <row r="77" spans="3:15" hidden="1">
       <c r="C77" t="s">
         <v>265</v>
       </c>
@@ -7486,7 +7527,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="78" spans="3:15">
+    <row r="78" spans="3:15" hidden="1">
       <c r="C78" t="s">
         <v>268</v>
       </c>
@@ -7527,7 +7568,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="3:15">
+    <row r="79" spans="3:15" hidden="1">
       <c r="C79" t="s">
         <v>271</v>
       </c>
@@ -7568,7 +7609,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="80" spans="3:15">
+    <row r="80" spans="3:15" hidden="1">
       <c r="C80" t="s">
         <v>274</v>
       </c>
@@ -7609,7 +7650,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="81" spans="3:15">
+    <row r="81" spans="3:15" hidden="1">
       <c r="C81" t="s">
         <v>277</v>
       </c>
@@ -7650,7 +7691,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="82" spans="3:15">
+    <row r="82" spans="3:15" hidden="1">
       <c r="C82" t="s">
         <v>280</v>
       </c>
@@ -7691,7 +7732,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="83" spans="3:15">
+    <row r="83" spans="3:15" hidden="1">
       <c r="C83" t="s">
         <v>283</v>
       </c>
@@ -7732,7 +7773,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="84" spans="3:15">
+    <row r="84" spans="3:15" hidden="1">
       <c r="C84" t="s">
         <v>286</v>
       </c>
@@ -7773,7 +7814,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="85" spans="3:15">
+    <row r="85" spans="3:15" hidden="1">
       <c r="C85" t="s">
         <v>289</v>
       </c>
@@ -7814,7 +7855,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="86" spans="3:15">
+    <row r="86" spans="3:15" hidden="1">
       <c r="C86" t="s">
         <v>292</v>
       </c>
@@ -7855,7 +7896,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="87" spans="3:15">
+    <row r="87" spans="3:15" hidden="1">
       <c r="C87" t="s">
         <v>295</v>
       </c>
@@ -7896,7 +7937,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="88" spans="3:15">
+    <row r="88" spans="3:15" hidden="1">
       <c r="C88" t="s">
         <v>298</v>
       </c>
@@ -7937,7 +7978,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="89" spans="3:15">
+    <row r="89" spans="3:15" hidden="1">
       <c r="C89" t="s">
         <v>301</v>
       </c>
@@ -7978,7 +8019,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="90" spans="3:15">
+    <row r="90" spans="3:15" hidden="1">
       <c r="C90" t="s">
         <v>304</v>
       </c>
@@ -8019,7 +8060,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="91" spans="3:15">
+    <row r="91" spans="3:15" hidden="1">
       <c r="C91" t="s">
         <v>304</v>
       </c>
@@ -8060,7 +8101,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="92" spans="3:15">
+    <row r="92" spans="3:15" hidden="1">
       <c r="C92" t="s">
         <v>309</v>
       </c>
@@ -8101,7 +8142,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="93" spans="3:15">
+    <row r="93" spans="3:15" hidden="1">
       <c r="C93" t="s">
         <v>309</v>
       </c>
@@ -8142,7 +8183,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="94" spans="3:15">
+    <row r="94" spans="3:15" hidden="1">
       <c r="C94" t="s">
         <v>312</v>
       </c>
@@ -8183,7 +8224,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="95" spans="3:15">
+    <row r="95" spans="3:15" hidden="1">
       <c r="C95" t="s">
         <v>315</v>
       </c>
@@ -8224,7 +8265,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="96" spans="3:15">
+    <row r="96" spans="3:15" hidden="1">
       <c r="C96" t="s">
         <v>318</v>
       </c>
@@ -8265,7 +8306,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="97" spans="3:15">
+    <row r="97" spans="3:15" hidden="1">
       <c r="C97" t="s">
         <v>321</v>
       </c>
@@ -8306,7 +8347,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="98" spans="3:15">
+    <row r="98" spans="3:15" hidden="1">
       <c r="C98" t="s">
         <v>324</v>
       </c>
@@ -8347,7 +8388,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="99" spans="3:15">
+    <row r="99" spans="3:15" hidden="1">
       <c r="C99" t="s">
         <v>327</v>
       </c>
@@ -8388,7 +8429,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="100" spans="3:15">
+    <row r="100" spans="3:15" hidden="1">
       <c r="C100" t="s">
         <v>330</v>
       </c>
@@ -8429,7 +8470,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="101" spans="3:15">
+    <row r="101" spans="3:15" hidden="1">
       <c r="C101" t="s">
         <v>333</v>
       </c>
@@ -8470,7 +8511,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="102" spans="3:15">
+    <row r="102" spans="3:15" hidden="1">
       <c r="C102" t="s">
         <v>333</v>
       </c>
@@ -8511,7 +8552,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="103" spans="3:15">
+    <row r="103" spans="3:15" hidden="1">
       <c r="C103" t="s">
         <v>336</v>
       </c>
@@ -8552,7 +8593,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="104" spans="3:15">
+    <row r="104" spans="3:15" hidden="1">
       <c r="C104" t="s">
         <v>339</v>
       </c>
@@ -8593,7 +8634,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="105" spans="3:15">
+    <row r="105" spans="3:15" hidden="1">
       <c r="C105" t="s">
         <v>342</v>
       </c>
@@ -8634,7 +8675,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="106" spans="3:15">
+    <row r="106" spans="3:15" hidden="1">
       <c r="C106" t="s">
         <v>345</v>
       </c>
@@ -8675,7 +8716,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="107" spans="3:15">
+    <row r="107" spans="3:15" hidden="1">
       <c r="C107" t="s">
         <v>348</v>
       </c>
@@ -8716,7 +8757,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="108" spans="3:15">
+    <row r="108" spans="3:15" hidden="1">
       <c r="C108" t="s">
         <v>351</v>
       </c>
@@ -8757,7 +8798,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="109" spans="3:15">
+    <row r="109" spans="3:15" hidden="1">
       <c r="C109" t="s">
         <v>354</v>
       </c>
@@ -8798,7 +8839,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="110" spans="3:15">
+    <row r="110" spans="3:15" hidden="1">
       <c r="C110" t="s">
         <v>354</v>
       </c>
@@ -8839,7 +8880,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="111" spans="3:15">
+    <row r="111" spans="3:15" hidden="1">
       <c r="C111" t="s">
         <v>357</v>
       </c>
@@ -8880,7 +8921,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="112" spans="3:15">
+    <row r="112" spans="3:15" hidden="1">
       <c r="C112" t="s">
         <v>360</v>
       </c>
@@ -8921,7 +8962,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="113" spans="3:15">
+    <row r="113" spans="3:15" hidden="1">
       <c r="C113" t="s">
         <v>363</v>
       </c>
@@ -8962,7 +9003,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="114" spans="3:15">
+    <row r="114" spans="3:15" hidden="1">
       <c r="C114" t="s">
         <v>366</v>
       </c>
@@ -9003,7 +9044,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="115" spans="3:15">
+    <row r="115" spans="3:15" hidden="1">
       <c r="C115" t="s">
         <v>366</v>
       </c>
@@ -9044,7 +9085,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="116" spans="3:15">
+    <row r="116" spans="3:15" hidden="1">
       <c r="C116" t="s">
         <v>369</v>
       </c>
@@ -9085,7 +9126,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="117" spans="3:15">
+    <row r="117" spans="3:15" hidden="1">
       <c r="C117" t="s">
         <v>372</v>
       </c>
@@ -9126,7 +9167,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="118" spans="3:15">
+    <row r="118" spans="3:15" hidden="1">
       <c r="C118" t="s">
         <v>375</v>
       </c>
@@ -9167,7 +9208,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="119" spans="3:15">
+    <row r="119" spans="3:15" hidden="1">
       <c r="C119" t="s">
         <v>378</v>
       </c>
@@ -9208,7 +9249,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="120" spans="3:15">
+    <row r="120" spans="3:15" hidden="1">
       <c r="C120" t="s">
         <v>381</v>
       </c>
@@ -9249,7 +9290,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="121" spans="3:15">
+    <row r="121" spans="3:15" hidden="1">
       <c r="C121" t="s">
         <v>384</v>
       </c>
@@ -9290,7 +9331,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="122" spans="3:15">
+    <row r="122" spans="3:15" hidden="1">
       <c r="C122" t="s">
         <v>387</v>
       </c>
@@ -9331,7 +9372,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="123" spans="3:15">
+    <row r="123" spans="3:15" hidden="1">
       <c r="C123" t="s">
         <v>390</v>
       </c>
@@ -9372,7 +9413,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="124" spans="3:15">
+    <row r="124" spans="3:15" hidden="1">
       <c r="C124" t="s">
         <v>393</v>
       </c>
@@ -9413,7 +9454,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="125" spans="3:15">
+    <row r="125" spans="3:15" hidden="1">
       <c r="C125" t="s">
         <v>396</v>
       </c>
@@ -9454,7 +9495,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="126" spans="3:15">
+    <row r="126" spans="3:15" hidden="1">
       <c r="C126" t="s">
         <v>399</v>
       </c>
@@ -9495,7 +9536,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="127" spans="3:15">
+    <row r="127" spans="3:15" hidden="1">
       <c r="C127" t="s">
         <v>402</v>
       </c>
@@ -9536,7 +9577,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="128" spans="3:15">
+    <row r="128" spans="3:15" hidden="1">
       <c r="C128" t="s">
         <v>405</v>
       </c>
@@ -9577,7 +9618,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="129" spans="3:15">
+    <row r="129" spans="3:15" hidden="1">
       <c r="C129" t="s">
         <v>408</v>
       </c>
@@ -9618,7 +9659,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="130" spans="3:15">
+    <row r="130" spans="3:15" hidden="1">
       <c r="C130" t="s">
         <v>411</v>
       </c>
@@ -9659,7 +9700,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="131" spans="3:15">
+    <row r="131" spans="3:15" hidden="1">
       <c r="C131" t="s">
         <v>414</v>
       </c>
@@ -9700,7 +9741,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="132" spans="3:15">
+    <row r="132" spans="3:15" hidden="1">
       <c r="C132" t="s">
         <v>417</v>
       </c>
@@ -9741,7 +9782,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="133" spans="3:15">
+    <row r="133" spans="3:15" hidden="1">
       <c r="C133" t="s">
         <v>420</v>
       </c>
@@ -9782,7 +9823,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="134" spans="3:15">
+    <row r="134" spans="3:15" hidden="1">
       <c r="C134" t="s">
         <v>420</v>
       </c>
@@ -9823,7 +9864,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="135" spans="3:15">
+    <row r="135" spans="3:15" hidden="1">
       <c r="C135" t="s">
         <v>425</v>
       </c>
@@ -9864,7 +9905,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="136" spans="3:15">
+    <row r="136" spans="3:15" hidden="1">
       <c r="C136" t="s">
         <v>428</v>
       </c>
@@ -9905,7 +9946,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="137" spans="3:15">
+    <row r="137" spans="3:15" hidden="1">
       <c r="C137" t="s">
         <v>431</v>
       </c>
@@ -9946,7 +9987,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="138" spans="3:15">
+    <row r="138" spans="3:15" hidden="1">
       <c r="C138" t="s">
         <v>434</v>
       </c>
@@ -9987,7 +10028,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="139" spans="3:15">
+    <row r="139" spans="3:15" hidden="1">
       <c r="C139" t="s">
         <v>437</v>
       </c>
@@ -10028,7 +10069,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="140" spans="3:15">
+    <row r="140" spans="3:15" hidden="1">
       <c r="C140" t="s">
         <v>440</v>
       </c>
@@ -10069,7 +10110,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="141" spans="3:15">
+    <row r="141" spans="3:15" hidden="1">
       <c r="C141" t="s">
         <v>443</v>
       </c>
@@ -10110,7 +10151,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="142" spans="3:15">
+    <row r="142" spans="3:15" hidden="1">
       <c r="C142" t="s">
         <v>446</v>
       </c>
@@ -10151,7 +10192,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="143" spans="3:15">
+    <row r="143" spans="3:15" hidden="1">
       <c r="C143" t="s">
         <v>446</v>
       </c>
@@ -10192,7 +10233,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="144" spans="3:15">
+    <row r="144" spans="3:15" hidden="1">
       <c r="C144" t="s">
         <v>449</v>
       </c>
@@ -10233,7 +10274,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="145" spans="3:15">
+    <row r="145" spans="3:15" hidden="1">
       <c r="C145" t="s">
         <v>452</v>
       </c>
@@ -10274,7 +10315,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="146" spans="3:15">
+    <row r="146" spans="3:15" hidden="1">
       <c r="C146" t="s">
         <v>455</v>
       </c>
@@ -10315,7 +10356,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="147" spans="3:15">
+    <row r="147" spans="3:15" hidden="1">
       <c r="C147" t="s">
         <v>458</v>
       </c>
@@ -10356,7 +10397,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="148" spans="3:15">
+    <row r="148" spans="3:15" hidden="1">
       <c r="C148" t="s">
         <v>458</v>
       </c>
@@ -10397,7 +10438,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="149" spans="3:15">
+    <row r="149" spans="3:15" hidden="1">
       <c r="C149" t="s">
         <v>463</v>
       </c>
@@ -10438,7 +10479,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="150" spans="3:15">
+    <row r="150" spans="3:15" hidden="1">
       <c r="C150" t="s">
         <v>466</v>
       </c>
@@ -10479,7 +10520,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="151" spans="3:15">
+    <row r="151" spans="3:15" hidden="1">
       <c r="C151" t="s">
         <v>469</v>
       </c>
@@ -10520,7 +10561,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="152" spans="3:15">
+    <row r="152" spans="3:15" hidden="1">
       <c r="C152" t="s">
         <v>472</v>
       </c>
@@ -10561,7 +10602,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="153" spans="3:15">
+    <row r="153" spans="3:15" hidden="1">
       <c r="C153" t="s">
         <v>475</v>
       </c>
@@ -10602,7 +10643,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="154" spans="3:15">
+    <row r="154" spans="3:15" hidden="1">
       <c r="C154" t="s">
         <v>475</v>
       </c>
@@ -10643,7 +10684,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="155" spans="3:15">
+    <row r="155" spans="3:15" hidden="1">
       <c r="C155" t="s">
         <v>478</v>
       </c>
@@ -10684,7 +10725,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="156" spans="3:15">
+    <row r="156" spans="3:15" hidden="1">
       <c r="C156" t="s">
         <v>481</v>
       </c>
@@ -10725,7 +10766,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="157" spans="3:15">
+    <row r="157" spans="3:15" hidden="1">
       <c r="C157" t="s">
         <v>484</v>
       </c>
@@ -10766,7 +10807,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="158" spans="3:15">
+    <row r="158" spans="3:15" hidden="1">
       <c r="C158" t="s">
         <v>484</v>
       </c>
@@ -10807,7 +10848,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="159" spans="3:15">
+    <row r="159" spans="3:15" hidden="1">
       <c r="C159" t="s">
         <v>487</v>
       </c>
@@ -10848,7 +10889,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="160" spans="3:15">
+    <row r="160" spans="3:15" hidden="1">
       <c r="C160" t="s">
         <v>490</v>
       </c>
@@ -10889,7 +10930,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="161" spans="3:15">
+    <row r="161" spans="3:15" hidden="1">
       <c r="C161" t="s">
         <v>491</v>
       </c>
@@ -10930,7 +10971,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="162" spans="3:15">
+    <row r="162" spans="3:15" hidden="1">
       <c r="C162" t="s">
         <v>494</v>
       </c>
@@ -10971,7 +11012,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="163" spans="3:15">
+    <row r="163" spans="3:15" hidden="1">
       <c r="C163" t="s">
         <v>497</v>
       </c>
@@ -11012,7 +11053,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="164" spans="3:15">
+    <row r="164" spans="3:15" hidden="1">
       <c r="C164" t="s">
         <v>500</v>
       </c>
@@ -11053,7 +11094,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="165" spans="3:15">
+    <row r="165" spans="3:15" hidden="1">
       <c r="C165" t="s">
         <v>503</v>
       </c>
@@ -11094,7 +11135,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="166" spans="3:15">
+    <row r="166" spans="3:15" hidden="1">
       <c r="C166" t="s">
         <v>503</v>
       </c>
@@ -11135,7 +11176,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="167" spans="3:15">
+    <row r="167" spans="3:15" hidden="1">
       <c r="C167" t="s">
         <v>506</v>
       </c>
@@ -11176,7 +11217,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="168" spans="3:15">
+    <row r="168" spans="3:15" hidden="1">
       <c r="C168" t="s">
         <v>506</v>
       </c>
@@ -11217,7 +11258,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="169" spans="3:15">
+    <row r="169" spans="3:15" hidden="1">
       <c r="C169" t="s">
         <v>509</v>
       </c>
@@ -11258,7 +11299,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="170" spans="3:15">
+    <row r="170" spans="3:15" hidden="1">
       <c r="C170" t="s">
         <v>512</v>
       </c>
@@ -11299,7 +11340,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="171" spans="3:15">
+    <row r="171" spans="3:15" hidden="1">
       <c r="C171" t="s">
         <v>515</v>
       </c>
@@ -11340,7 +11381,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="172" spans="3:15">
+    <row r="172" spans="3:15" hidden="1">
       <c r="C172" t="s">
         <v>518</v>
       </c>
@@ -11381,7 +11422,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="173" spans="3:15">
+    <row r="173" spans="3:15" hidden="1">
       <c r="C173" t="s">
         <v>521</v>
       </c>
@@ -11422,7 +11463,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="174" spans="3:15">
+    <row r="174" spans="3:15" hidden="1">
       <c r="C174" t="s">
         <v>524</v>
       </c>
@@ -11463,7 +11504,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="175" spans="3:15">
+    <row r="175" spans="3:15" hidden="1">
       <c r="C175" t="s">
         <v>524</v>
       </c>
@@ -11504,7 +11545,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="176" spans="3:15">
+    <row r="176" spans="3:15" hidden="1">
       <c r="C176" t="s">
         <v>528</v>
       </c>
@@ -11545,7 +11586,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="177" spans="3:15">
+    <row r="177" spans="3:15" hidden="1">
       <c r="C177" t="s">
         <v>532</v>
       </c>
@@ -11586,7 +11627,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="178" spans="3:15">
+    <row r="178" spans="3:15" hidden="1">
       <c r="C178" t="s">
         <v>535</v>
       </c>
@@ -11627,7 +11668,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="179" spans="3:15">
+    <row r="179" spans="3:15" hidden="1">
       <c r="C179" t="s">
         <v>535</v>
       </c>
@@ -11668,7 +11709,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="180" spans="3:15">
+    <row r="180" spans="3:15" hidden="1">
       <c r="C180" t="s">
         <v>538</v>
       </c>
@@ -11709,7 +11750,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="181" spans="3:15">
+    <row r="181" spans="3:15" hidden="1">
       <c r="C181" t="s">
         <v>541</v>
       </c>
@@ -11750,7 +11791,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="182" spans="3:15">
+    <row r="182" spans="3:15" hidden="1">
       <c r="C182" t="s">
         <v>542</v>
       </c>
@@ -11791,7 +11832,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="183" spans="3:15">
+    <row r="183" spans="3:15" hidden="1">
       <c r="C183" t="s">
         <v>545</v>
       </c>
@@ -11832,7 +11873,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="184" spans="3:15">
+    <row r="184" spans="3:15" hidden="1">
       <c r="C184" t="s">
         <v>548</v>
       </c>
@@ -11873,7 +11914,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="185" spans="3:15">
+    <row r="185" spans="3:15" hidden="1">
       <c r="C185" t="s">
         <v>548</v>
       </c>
@@ -11914,7 +11955,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="186" spans="3:15">
+    <row r="186" spans="3:15" hidden="1">
       <c r="C186" t="s">
         <v>551</v>
       </c>
@@ -11955,7 +11996,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="187" spans="3:15">
+    <row r="187" spans="3:15" hidden="1">
       <c r="C187" t="s">
         <v>551</v>
       </c>
@@ -11996,7 +12037,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="188" spans="3:15">
+    <row r="188" spans="3:15" hidden="1">
       <c r="C188" t="s">
         <v>556</v>
       </c>
@@ -12037,7 +12078,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="189" spans="3:15">
+    <row r="189" spans="3:15" hidden="1">
       <c r="C189" t="s">
         <v>559</v>
       </c>
@@ -12078,7 +12119,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="190" spans="3:15">
+    <row r="190" spans="3:15" hidden="1">
       <c r="C190" t="s">
         <v>562</v>
       </c>
@@ -12119,7 +12160,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="191" spans="3:15">
+    <row r="191" spans="3:15" hidden="1">
       <c r="C191" t="s">
         <v>565</v>
       </c>
@@ -12160,7 +12201,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="192" spans="3:15">
+    <row r="192" spans="3:15" hidden="1">
       <c r="C192" t="s">
         <v>568</v>
       </c>
@@ -12201,7 +12242,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="193" spans="3:15">
+    <row r="193" spans="3:15" hidden="1">
       <c r="C193" t="s">
         <v>571</v>
       </c>
@@ -12242,7 +12283,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="3:15">
+    <row r="194" spans="3:15" hidden="1">
       <c r="C194" t="s">
         <v>574</v>
       </c>
@@ -12283,7 +12324,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="195" spans="3:15">
+    <row r="195" spans="3:15" hidden="1">
       <c r="C195" t="s">
         <v>574</v>
       </c>
@@ -12324,7 +12365,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="196" spans="3:15">
+    <row r="196" spans="3:15" hidden="1">
       <c r="C196" t="s">
         <v>576</v>
       </c>
@@ -12365,7 +12406,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="197" spans="3:15">
+    <row r="197" spans="3:15" hidden="1">
       <c r="C197" t="s">
         <v>579</v>
       </c>
@@ -12406,7 +12447,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="198" spans="3:15">
+    <row r="198" spans="3:15" hidden="1">
       <c r="C198" t="s">
         <v>582</v>
       </c>
@@ -12447,7 +12488,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="199" spans="3:15">
+    <row r="199" spans="3:15" hidden="1">
       <c r="C199" t="s">
         <v>585</v>
       </c>
@@ -12488,7 +12529,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="200" spans="3:15">
+    <row r="200" spans="3:15" hidden="1">
       <c r="C200" t="s">
         <v>588</v>
       </c>
@@ -12529,7 +12570,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="201" spans="3:15">
+    <row r="201" spans="3:15" hidden="1">
       <c r="C201" t="s">
         <v>591</v>
       </c>
@@ -12570,7 +12611,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="202" spans="3:15">
+    <row r="202" spans="3:15" hidden="1">
       <c r="C202" t="s">
         <v>594</v>
       </c>
@@ -12611,7 +12652,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="203" spans="3:15">
+    <row r="203" spans="3:15" hidden="1">
       <c r="C203" t="s">
         <v>596</v>
       </c>
@@ -12652,7 +12693,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="204" spans="3:15">
+    <row r="204" spans="3:15" hidden="1">
       <c r="C204" t="s">
         <v>599</v>
       </c>
@@ -12693,7 +12734,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="205" spans="3:15">
+    <row r="205" spans="3:15" hidden="1">
       <c r="C205" t="s">
         <v>602</v>
       </c>
@@ -12734,7 +12775,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="206" spans="3:15">
+    <row r="206" spans="3:15" hidden="1">
       <c r="C206" t="s">
         <v>602</v>
       </c>
@@ -12775,7 +12816,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="207" spans="3:15">
+    <row r="207" spans="3:15" hidden="1">
       <c r="C207" t="s">
         <v>605</v>
       </c>
@@ -12816,7 +12857,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="208" spans="3:15">
+    <row r="208" spans="3:15" hidden="1">
       <c r="C208" t="s">
         <v>608</v>
       </c>
@@ -12857,7 +12898,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="209" spans="3:15">
+    <row r="209" spans="3:15" hidden="1">
       <c r="C209" t="s">
         <v>611</v>
       </c>
@@ -12898,7 +12939,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="210" spans="3:15">
+    <row r="210" spans="3:15" hidden="1">
       <c r="C210" t="s">
         <v>614</v>
       </c>
@@ -12939,7 +12980,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="211" spans="3:15">
+    <row r="211" spans="3:15" hidden="1">
       <c r="C211" t="s">
         <v>617</v>
       </c>
@@ -12980,7 +13021,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="212" spans="3:15">
+    <row r="212" spans="3:15" hidden="1">
       <c r="C212" t="s">
         <v>620</v>
       </c>
@@ -13021,7 +13062,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="213" spans="3:15">
+    <row r="213" spans="3:15" hidden="1">
       <c r="C213" t="s">
         <v>623</v>
       </c>
@@ -13062,7 +13103,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="214" spans="3:15">
+    <row r="214" spans="3:15" hidden="1">
       <c r="C214" t="s">
         <v>626</v>
       </c>
@@ -13103,7 +13144,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="215" spans="3:15">
+    <row r="215" spans="3:15" hidden="1">
       <c r="C215" t="s">
         <v>629</v>
       </c>
@@ -13144,7 +13185,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="216" spans="3:15">
+    <row r="216" spans="3:15" hidden="1">
       <c r="C216" t="s">
         <v>629</v>
       </c>
@@ -13185,7 +13226,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="217" spans="3:15">
+    <row r="217" spans="3:15" hidden="1">
       <c r="C217" t="s">
         <v>634</v>
       </c>
@@ -13226,7 +13267,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="218" spans="3:15">
+    <row r="218" spans="3:15" hidden="1">
       <c r="C218" t="s">
         <v>637</v>
       </c>
@@ -13267,7 +13308,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="219" spans="3:15">
+    <row r="219" spans="3:15" hidden="1">
       <c r="C219" t="s">
         <v>640</v>
       </c>
@@ -13308,7 +13349,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="220" spans="3:15">
+    <row r="220" spans="3:15" hidden="1">
       <c r="C220" t="s">
         <v>643</v>
       </c>
@@ -13349,7 +13390,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="221" spans="3:15">
+    <row r="221" spans="3:15" hidden="1">
       <c r="C221" t="s">
         <v>646</v>
       </c>
@@ -13390,7 +13431,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="222" spans="3:15">
+    <row r="222" spans="3:15" hidden="1">
       <c r="C222" t="s">
         <v>649</v>
       </c>
@@ -13431,7 +13472,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="223" spans="3:15">
+    <row r="223" spans="3:15" hidden="1">
       <c r="C223" t="s">
         <v>649</v>
       </c>
@@ -13472,7 +13513,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="224" spans="3:15">
+    <row r="224" spans="3:15" hidden="1">
       <c r="C224" t="s">
         <v>652</v>
       </c>
@@ -13513,7 +13554,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="225" spans="3:15">
+    <row r="225" spans="3:15" hidden="1">
       <c r="C225" t="s">
         <v>655</v>
       </c>
@@ -13554,7 +13595,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="226" spans="3:15">
+    <row r="226" spans="3:15" hidden="1">
       <c r="C226" t="s">
         <v>658</v>
       </c>
@@ -13595,7 +13636,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="227" spans="3:15">
+    <row r="227" spans="3:15" hidden="1">
       <c r="C227" t="s">
         <v>662</v>
       </c>
@@ -13636,7 +13677,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="228" spans="3:15">
+    <row r="228" spans="3:15" hidden="1">
       <c r="C228" t="s">
         <v>662</v>
       </c>
@@ -13677,7 +13718,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="229" spans="3:15">
+    <row r="229" spans="3:15" hidden="1">
       <c r="C229" t="s">
         <v>665</v>
       </c>
@@ -13718,7 +13759,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="230" spans="3:15">
+    <row r="230" spans="3:15" hidden="1">
       <c r="C230" t="s">
         <v>668</v>
       </c>
@@ -13759,7 +13800,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="231" spans="3:15">
+    <row r="231" spans="3:15" hidden="1">
       <c r="C231" t="s">
         <v>668</v>
       </c>
@@ -13800,7 +13841,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="232" spans="3:15">
+    <row r="232" spans="3:15" hidden="1">
       <c r="C232" t="s">
         <v>671</v>
       </c>
@@ -13841,7 +13882,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="233" spans="3:15">
+    <row r="233" spans="3:15" hidden="1">
       <c r="C233" t="s">
         <v>674</v>
       </c>
@@ -13882,7 +13923,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="234" spans="3:15">
+    <row r="234" spans="3:15" hidden="1">
       <c r="C234" t="s">
         <v>677</v>
       </c>
@@ -13923,7 +13964,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="235" spans="3:15">
+    <row r="235" spans="3:15" hidden="1">
       <c r="C235" t="s">
         <v>680</v>
       </c>
@@ -13964,7 +14005,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="236" spans="3:15">
+    <row r="236" spans="3:15" hidden="1">
       <c r="C236" t="s">
         <v>683</v>
       </c>
@@ -14005,7 +14046,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="237" spans="3:15">
+    <row r="237" spans="3:15" hidden="1">
       <c r="C237" t="s">
         <v>686</v>
       </c>
@@ -14046,7 +14087,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="238" spans="3:15">
+    <row r="238" spans="3:15" hidden="1">
       <c r="C238" t="s">
         <v>689</v>
       </c>
@@ -14087,7 +14128,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="239" spans="3:15">
+    <row r="239" spans="3:15" hidden="1">
       <c r="C239" t="s">
         <v>692</v>
       </c>
@@ -14128,7 +14169,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="240" spans="3:15">
+    <row r="240" spans="3:15" hidden="1">
       <c r="C240" t="s">
         <v>695</v>
       </c>
@@ -14169,7 +14210,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="241" spans="3:15">
+    <row r="241" spans="3:15" hidden="1">
       <c r="C241" t="s">
         <v>695</v>
       </c>
@@ -14210,7 +14251,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="242" spans="3:15">
+    <row r="242" spans="3:15" hidden="1">
       <c r="C242" t="s">
         <v>698</v>
       </c>
@@ -14251,7 +14292,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="243" spans="3:15">
+    <row r="243" spans="3:15" hidden="1">
       <c r="C243" t="s">
         <v>701</v>
       </c>
@@ -14292,7 +14333,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="244" spans="3:15">
+    <row r="244" spans="3:15" hidden="1">
       <c r="C244" t="s">
         <v>701</v>
       </c>
@@ -14333,7 +14374,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="245" spans="3:15">
+    <row r="245" spans="3:15" hidden="1">
       <c r="C245" t="s">
         <v>704</v>
       </c>
@@ -14374,7 +14415,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="246" spans="3:15">
+    <row r="246" spans="3:15" hidden="1">
       <c r="C246" t="s">
         <v>707</v>
       </c>
@@ -14415,7 +14456,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="247" spans="3:15">
+    <row r="247" spans="3:15" hidden="1">
       <c r="C247" t="s">
         <v>710</v>
       </c>
@@ -14456,7 +14497,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="248" spans="3:15">
+    <row r="248" spans="3:15" hidden="1">
       <c r="C248" t="s">
         <v>713</v>
       </c>
@@ -14497,7 +14538,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="249" spans="3:15">
+    <row r="249" spans="3:15" hidden="1">
       <c r="C249" t="s">
         <v>716</v>
       </c>
@@ -14538,7 +14579,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="250" spans="3:15">
+    <row r="250" spans="3:15" hidden="1">
       <c r="C250" t="s">
         <v>719</v>
       </c>
@@ -14579,7 +14620,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="251" spans="3:15">
+    <row r="251" spans="3:15" hidden="1">
       <c r="C251" t="s">
         <v>722</v>
       </c>
@@ -14620,7 +14661,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="252" spans="3:15">
+    <row r="252" spans="3:15" hidden="1">
       <c r="C252" t="s">
         <v>725</v>
       </c>
@@ -14661,7 +14702,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="253" spans="3:15">
+    <row r="253" spans="3:15" hidden="1">
       <c r="C253" t="s">
         <v>725</v>
       </c>
@@ -14702,7 +14743,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="254" spans="3:15">
+    <row r="254" spans="3:15" hidden="1">
       <c r="C254" t="s">
         <v>728</v>
       </c>
@@ -14743,7 +14784,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="255" spans="3:15">
+    <row r="255" spans="3:15" hidden="1">
       <c r="C255" t="s">
         <v>728</v>
       </c>
@@ -14784,7 +14825,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="256" spans="3:15">
+    <row r="256" spans="3:15" hidden="1">
       <c r="C256" t="s">
         <v>733</v>
       </c>
@@ -14825,7 +14866,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="257" spans="3:15">
+    <row r="257" spans="3:15" hidden="1">
       <c r="C257" t="s">
         <v>736</v>
       </c>
@@ -14866,7 +14907,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="258" spans="3:15">
+    <row r="258" spans="3:15" hidden="1">
       <c r="C258" t="s">
         <v>739</v>
       </c>
@@ -14907,7 +14948,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="259" spans="3:15">
+    <row r="259" spans="3:15" hidden="1">
       <c r="C259" t="s">
         <v>739</v>
       </c>
@@ -14948,7 +14989,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="260" spans="3:15">
+    <row r="260" spans="3:15" hidden="1">
       <c r="C260" t="s">
         <v>744</v>
       </c>
@@ -14989,7 +15030,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="261" spans="3:15">
+    <row r="261" spans="3:15" hidden="1">
       <c r="C261" t="s">
         <v>747</v>
       </c>
@@ -15030,7 +15071,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="262" spans="3:15">
+    <row r="262" spans="3:15" hidden="1">
       <c r="C262" t="s">
         <v>750</v>
       </c>
@@ -15071,7 +15112,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="263" spans="3:15">
+    <row r="263" spans="3:15" hidden="1">
       <c r="C263" t="s">
         <v>753</v>
       </c>
@@ -15112,7 +15153,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="264" spans="3:15">
+    <row r="264" spans="3:15" hidden="1">
       <c r="C264" t="s">
         <v>756</v>
       </c>
@@ -15153,7 +15194,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="265" spans="3:15">
+    <row r="265" spans="3:15" hidden="1">
       <c r="C265" t="s">
         <v>759</v>
       </c>
@@ -15194,7 +15235,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="266" spans="3:15">
+    <row r="266" spans="3:15" hidden="1">
       <c r="C266" t="s">
         <v>762</v>
       </c>
@@ -15235,7 +15276,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="267" spans="3:15">
+    <row r="267" spans="3:15" hidden="1">
       <c r="C267" t="s">
         <v>765</v>
       </c>
@@ -18941,4 +18982,455 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{056D4C31-6BF7-4F39-B5EE-B0BC201D12D6}">
+  <dimension ref="A4:C22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="28.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:3">
+      <c r="B4" s="28" t="s">
+        <v>780</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="str">
+        <f>IFERROR(VLOOKUP($C$4,staff[],A6,FALSE),"Not Found")</f>
+        <v>Edd</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="str">
+        <f>IFERROR(VLOOKUP($C$4,staff[],A7,FALSE),"Not Found")</f>
+        <v>MacKnockiter</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="str">
+        <f>IFERROR(VLOOKUP($C$4,staff[],A8,FALSE),"Not Found")</f>
+        <v>Accounting</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9">
+        <f>IFERROR(VLOOKUP($C$4,staff[],A9,FALSE),"Not Found")</f>
+        <v>119022.49</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="C18">
+        <f>MATCH(C17,staff[Last Name],0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="34" t="s">
+        <v>780</v>
+      </c>
+      <c r="C20" t="str">
+        <f>INDEX(staff[Emp ID],MATCH(C17,staff[Last Name],0))</f>
+        <v>PR00113</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="str">
+        <f>INDEX(staff[Department],MATCH(C17,staff[Last Name],0))</f>
+        <v>Business Development</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <f>INDEX(staff[Salary],MATCH(C17,staff[Last Name],0))</f>
+        <v>80695.740000000005</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46536243-F308-454E-A744-58FF22B55FB4}">
+  <dimension ref="B4:N44"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:3">
+      <c r="B4" s="28" t="s">
+        <v>781</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" t="s">
+        <v>782</v>
+      </c>
+      <c r="C6" t="str">
+        <f>_xlfn.XLOOKUP(C4,staff[Emp ID],staff[First Name],"Not Found")</f>
+        <v>Edd</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" t="s">
+        <v>783</v>
+      </c>
+      <c r="C7" t="str">
+        <f>_xlfn.XLOOKUP(C4,staff[Emp ID],staff[Last Name],"Not Found")</f>
+        <v>MacKnockiter</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="str">
+        <f>_xlfn.XLOOKUP(C4,staff[Emp ID],staff[Department],"Not Found")</f>
+        <v>Accounting</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3">
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9">
+        <f>_xlfn.XLOOKUP(C4,staff[Emp ID],staff[Salary],"Not Found")</f>
+        <v>119022.49</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3">
+      <c r="B14" s="28" t="s">
+        <v>783</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14">
+      <c r="B17" s="34" t="s">
+        <v>781</v>
+      </c>
+      <c r="C17" t="str">
+        <f>_xlfn.XLOOKUP(C14,staff[Last Name],staff[Emp ID],"Not Found")</f>
+        <v>PR00113</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14">
+      <c r="B18" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="str">
+        <f>_xlfn.XLOOKUP(C14,staff[Last Name],staff[Department],"Not Found")</f>
+        <v>Business Development</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14">
+      <c r="B19" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <f>_xlfn.XLOOKUP(C14,staff[Last Name],staff[Salary],"Not Found")</f>
+        <v>80695.740000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14">
+      <c r="B22" s="34" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14">
+      <c r="B23" t="str" cm="1">
+        <f t="array" ref="B23:N23">_xlfn.XLOOKUP(C14,staff[Last Name],staff[],"Not Found")</f>
+        <v>PR00113</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Van</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Tuxwell</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Female</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Business Development</v>
+      </c>
+      <c r="G23">
+        <v>80695.740000000005</v>
+      </c>
+      <c r="H23" t="str">
+        <v>50k to 100k</v>
+      </c>
+      <c r="I23">
+        <v>43360</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Columbus, USA</v>
+      </c>
+      <c r="M23">
+        <v>5.7643835616438359</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Full time</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14">
+      <c r="B25" s="34" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14">
+      <c r="B26" t="str" cm="1">
+        <f t="array" ref="B26:B38">TRANSPOSE(_xlfn.XLOOKUP(C14,staff[Last Name],staff[],"Not Found"))</f>
+        <v>PR00113</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14">
+      <c r="B27" t="str">
+        <v>Van</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14">
+      <c r="B28" t="str">
+        <v>Tuxwell</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14">
+      <c r="B29" t="str">
+        <v>Female</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14">
+      <c r="B30" t="str">
+        <v>Business Development</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14">
+      <c r="B31">
+        <v>80695.740000000005</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14">
+      <c r="B32" t="str">
+        <v>50k to 100k</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14">
+      <c r="B33">
+        <v>43360</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14">
+      <c r="B34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:14">
+      <c r="B35" t="str">
+        <v>Permanent</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14">
+      <c r="B36" t="str">
+        <v>Columbus, USA</v>
+      </c>
+    </row>
+    <row r="37" spans="2:14">
+      <c r="B37">
+        <v>5.7643835616438359</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14">
+      <c r="B38" t="str">
+        <v>Full time</v>
+      </c>
+    </row>
+    <row r="41" spans="2:14" ht="30.75">
+      <c r="B41" s="36" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14">
+      <c r="B42" t="str" cm="1">
+        <f t="array" ref="B42:N44">_xlfn._xlws.FILTER(staff[], staff[Last Name]=C14)</f>
+        <v>PR00113</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Van</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Tuxwell</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Female</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Business Development</v>
+      </c>
+      <c r="G42">
+        <v>80695.740000000005</v>
+      </c>
+      <c r="H42" t="str">
+        <v>50k to 100k</v>
+      </c>
+      <c r="I42">
+        <v>43360</v>
+      </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Columbus, USA</v>
+      </c>
+      <c r="M42">
+        <v>5.7643835616438359</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Full time</v>
+      </c>
+    </row>
+    <row r="43" spans="2:14">
+      <c r="B43" t="str">
+        <v>PR00113</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Van</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Tuxwell</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Female</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Business Development</v>
+      </c>
+      <c r="G43">
+        <v>80695.740000000005</v>
+      </c>
+      <c r="H43" t="str">
+        <v>50k to 100k</v>
+      </c>
+      <c r="I43">
+        <v>43360</v>
+      </c>
+      <c r="J43">
+        <v>1</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Columbus, USA</v>
+      </c>
+      <c r="M43">
+        <v>5.7643835616438359</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Full time</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14">
+      <c r="B44" t="str">
+        <v>PR04380</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Van</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Tuxwell</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Female</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Business Development</v>
+      </c>
+      <c r="G44">
+        <v>80695.740000000005</v>
+      </c>
+      <c r="H44" t="str">
+        <v>50k to 100k</v>
+      </c>
+      <c r="I44">
+        <v>43787</v>
+      </c>
+      <c r="J44">
+        <v>0.8</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Columbus, USA</v>
+      </c>
+      <c r="M44">
+        <v>4.5945205479452058</v>
+      </c>
+      <c r="N44" t="str">
+        <v>Part time</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>